<commit_message>
Criação da view para importação de dados Exel
</commit_message>
<xml_diff>
--- a/Dados Integrador/temperatura.xlsx
+++ b/Dados Integrador/temperatura.xlsx
@@ -820,7 +820,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="3" t="s">
         <v>6</v>
       </c>
@@ -840,7 +840,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="3" t="s">
         <v>6</v>
       </c>
@@ -860,7 +860,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="3" t="s">
         <v>6</v>
       </c>
@@ -880,7 +880,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="3" t="s">
         <v>6</v>
       </c>
@@ -900,7 +900,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="3" t="s">
         <v>6</v>
       </c>
@@ -920,7 +920,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="3" t="s">
         <v>6</v>
       </c>
@@ -940,7 +940,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="3" t="s">
         <v>6</v>
       </c>
@@ -960,7 +960,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="3" t="s">
         <v>6</v>
       </c>

</xml_diff>